<commit_message>
Update date format and cell format
</commit_message>
<xml_diff>
--- a/public/AxisBank_Payout_Verification.xlsx
+++ b/public/AxisBank_Payout_Verification.xlsx
@@ -32,8 +32,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="60" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -67,7 +68,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -374,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE53"/>
+  <dimension ref="A1:AF53"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="29"/>
     <col min="2" max="2" customWidth="1" width="29"/>
@@ -555,7 +556,7 @@
         <v>SBIN0002571</v>
       </c>
       <c r="G2" s="2" t="str">
-        <v>09/05/2026</v>
+        <v>05/09/2026</v>
       </c>
       <c r="H2" t="str">
         <v>N</v>
@@ -627,6 +628,9 @@
         <v/>
       </c>
       <c r="AE2" t="str">
+        <v/>
+      </c>
+      <c r="AF2" t="str">
         <v/>
       </c>
     </row>
@@ -649,8 +653,8 @@
       <c r="F3" t="str">
         <v>BKID0000083</v>
       </c>
-      <c r="G3" t="str">
-        <v>09/05/2026</v>
+      <c r="G3" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H3" t="str">
         <v>N</v>
@@ -722,6 +726,9 @@
         <v/>
       </c>
       <c r="AE3" t="str">
+        <v/>
+      </c>
+      <c r="AF3" t="str">
         <v/>
       </c>
     </row>
@@ -744,8 +751,8 @@
       <c r="F4" t="str">
         <v>SBIN0005794</v>
       </c>
-      <c r="G4" t="str">
-        <v>09/05/2026</v>
+      <c r="G4" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H4" t="str">
         <v>N</v>
@@ -817,6 +824,9 @@
         <v/>
       </c>
       <c r="AE4" t="str">
+        <v/>
+      </c>
+      <c r="AF4" t="str">
         <v/>
       </c>
     </row>
@@ -839,8 +849,8 @@
       <c r="F5" t="str">
         <v>HDFC0000485</v>
       </c>
-      <c r="G5" t="str">
-        <v>09/05/2026</v>
+      <c r="G5" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H5" t="str">
         <v>N</v>
@@ -912,6 +922,9 @@
         <v/>
       </c>
       <c r="AE5" t="str">
+        <v/>
+      </c>
+      <c r="AF5" t="str">
         <v/>
       </c>
     </row>
@@ -934,8 +947,8 @@
       <c r="F6" t="str">
         <v>HDFC0002870</v>
       </c>
-      <c r="G6" t="str">
-        <v>09/05/2026</v>
+      <c r="G6" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H6" t="str">
         <v>N</v>
@@ -1007,6 +1020,9 @@
         <v/>
       </c>
       <c r="AE6" t="str">
+        <v/>
+      </c>
+      <c r="AF6" t="str">
         <v/>
       </c>
     </row>
@@ -1029,8 +1045,8 @@
       <c r="F7" t="str">
         <v>HDFC0000729</v>
       </c>
-      <c r="G7" t="str">
-        <v>09/05/2026</v>
+      <c r="G7" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H7" t="str">
         <v>N</v>
@@ -1102,6 +1118,9 @@
         <v/>
       </c>
       <c r="AE7" t="str">
+        <v/>
+      </c>
+      <c r="AF7" t="str">
         <v/>
       </c>
     </row>
@@ -1124,8 +1143,8 @@
       <c r="F8" t="str">
         <v>UTIB0000029</v>
       </c>
-      <c r="G8" t="str">
-        <v>09/05/2026</v>
+      <c r="G8" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H8" t="str">
         <v>I</v>
@@ -1197,6 +1216,9 @@
         <v/>
       </c>
       <c r="AE8" t="str">
+        <v/>
+      </c>
+      <c r="AF8" t="str">
         <v/>
       </c>
     </row>
@@ -1219,8 +1241,8 @@
       <c r="F9" t="str">
         <v>JIOP0000001</v>
       </c>
-      <c r="G9" t="str">
-        <v>09/05/2026</v>
+      <c r="G9" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H9" t="str">
         <v>N</v>
@@ -1292,6 +1314,9 @@
         <v/>
       </c>
       <c r="AE9" t="str">
+        <v/>
+      </c>
+      <c r="AF9" t="str">
         <v/>
       </c>
     </row>
@@ -1314,8 +1339,8 @@
       <c r="F10" t="str">
         <v>JIOP0000001</v>
       </c>
-      <c r="G10" t="str">
-        <v>09/05/2026</v>
+      <c r="G10" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H10" t="str">
         <v>N</v>
@@ -1387,6 +1412,9 @@
         <v/>
       </c>
       <c r="AE10" t="str">
+        <v/>
+      </c>
+      <c r="AF10" t="str">
         <v/>
       </c>
     </row>
@@ -1409,8 +1437,8 @@
       <c r="F11" t="str">
         <v>HDFC0000729</v>
       </c>
-      <c r="G11" t="str">
-        <v>09/05/2026</v>
+      <c r="G11" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H11" t="str">
         <v>N</v>
@@ -1482,6 +1510,9 @@
         <v/>
       </c>
       <c r="AE11" t="str">
+        <v/>
+      </c>
+      <c r="AF11" t="str">
         <v/>
       </c>
     </row>
@@ -1504,8 +1535,8 @@
       <c r="F12" t="str">
         <v>SBIN0005794</v>
       </c>
-      <c r="G12" t="str">
-        <v>09/05/2026</v>
+      <c r="G12" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H12" t="str">
         <v>N</v>
@@ -1577,6 +1608,9 @@
         <v/>
       </c>
       <c r="AE12" t="str">
+        <v/>
+      </c>
+      <c r="AF12" t="str">
         <v/>
       </c>
     </row>
@@ -1599,8 +1633,8 @@
       <c r="F13" t="str">
         <v>ICIC0000946</v>
       </c>
-      <c r="G13" t="str">
-        <v>09/05/2026</v>
+      <c r="G13" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H13" t="str">
         <v>N</v>
@@ -1672,6 +1706,9 @@
         <v/>
       </c>
       <c r="AE13" t="str">
+        <v/>
+      </c>
+      <c r="AF13" t="str">
         <v/>
       </c>
     </row>
@@ -1694,8 +1731,8 @@
       <c r="F14" t="str">
         <v>CNRB0013128</v>
       </c>
-      <c r="G14" t="str">
-        <v>09/05/2026</v>
+      <c r="G14" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H14" t="str">
         <v>N</v>
@@ -1767,6 +1804,9 @@
         <v/>
       </c>
       <c r="AE14" t="str">
+        <v/>
+      </c>
+      <c r="AF14" t="str">
         <v/>
       </c>
     </row>
@@ -1789,8 +1829,8 @@
       <c r="F15" t="str">
         <v>CNRB0013128</v>
       </c>
-      <c r="G15" t="str">
-        <v>09/05/2026</v>
+      <c r="G15" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H15" t="str">
         <v>R</v>
@@ -1862,6 +1902,9 @@
         <v/>
       </c>
       <c r="AE15" t="str">
+        <v/>
+      </c>
+      <c r="AF15" t="str">
         <v/>
       </c>
     </row>
@@ -1884,8 +1927,8 @@
       <c r="F16" t="str">
         <v>CNRB0013128</v>
       </c>
-      <c r="G16" t="str">
-        <v>09/05/2026</v>
+      <c r="G16" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H16" t="str">
         <v>R</v>
@@ -1957,6 +2000,9 @@
         <v/>
       </c>
       <c r="AE16" t="str">
+        <v/>
+      </c>
+      <c r="AF16" t="str">
         <v/>
       </c>
     </row>
@@ -1979,8 +2025,8 @@
       <c r="F17" t="str">
         <v>CNRB0013128</v>
       </c>
-      <c r="G17" t="str">
-        <v>09/05/2026</v>
+      <c r="G17" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H17" t="str">
         <v>R</v>
@@ -2052,6 +2098,9 @@
         <v/>
       </c>
       <c r="AE17" t="str">
+        <v/>
+      </c>
+      <c r="AF17" t="str">
         <v/>
       </c>
     </row>
@@ -2074,8 +2123,8 @@
       <c r="F18" t="str">
         <v>SBIN00CARDS</v>
       </c>
-      <c r="G18" t="str">
-        <v>09/05/2026</v>
+      <c r="G18" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H18" t="str">
         <v>N</v>
@@ -2147,6 +2196,9 @@
         <v/>
       </c>
       <c r="AE18" t="str">
+        <v/>
+      </c>
+      <c r="AF18" t="str">
         <v/>
       </c>
     </row>
@@ -2169,8 +2221,8 @@
       <c r="F19" t="str">
         <v>HDFC0002578</v>
       </c>
-      <c r="G19" t="str">
-        <v>09/05/2026</v>
+      <c r="G19" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H19" t="str">
         <v>N</v>
@@ -2242,6 +2294,9 @@
         <v/>
       </c>
       <c r="AE19" t="str">
+        <v/>
+      </c>
+      <c r="AF19" t="str">
         <v/>
       </c>
     </row>
@@ -2264,8 +2319,8 @@
       <c r="F20" t="str">
         <v>ICIC0000946</v>
       </c>
-      <c r="G20" t="str">
-        <v>09/05/2026</v>
+      <c r="G20" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H20" t="str">
         <v>N</v>
@@ -2337,6 +2392,9 @@
         <v/>
       </c>
       <c r="AE20" t="str">
+        <v/>
+      </c>
+      <c r="AF20" t="str">
         <v/>
       </c>
     </row>
@@ -2359,8 +2417,8 @@
       <c r="F21" t="str">
         <v>ICIC0000946</v>
       </c>
-      <c r="G21" t="str">
-        <v>09/05/2026</v>
+      <c r="G21" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H21" t="str">
         <v>N</v>
@@ -2432,6 +2490,9 @@
         <v/>
       </c>
       <c r="AE21" t="str">
+        <v/>
+      </c>
+      <c r="AF21" t="str">
         <v/>
       </c>
     </row>
@@ -2454,8 +2515,8 @@
       <c r="F22" t="str">
         <v>HDFC0002578</v>
       </c>
-      <c r="G22" t="str">
-        <v>09/05/2026</v>
+      <c r="G22" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H22" t="str">
         <v>N</v>
@@ -2527,6 +2588,9 @@
         <v/>
       </c>
       <c r="AE22" t="str">
+        <v/>
+      </c>
+      <c r="AF22" t="str">
         <v/>
       </c>
     </row>
@@ -2549,8 +2613,8 @@
       <c r="F23" t="str">
         <v>SBIN0000055</v>
       </c>
-      <c r="G23" t="str">
-        <v>09/05/2026</v>
+      <c r="G23" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H23" t="str">
         <v>N</v>
@@ -2622,6 +2686,9 @@
         <v/>
       </c>
       <c r="AE23" t="str">
+        <v/>
+      </c>
+      <c r="AF23" t="str">
         <v/>
       </c>
     </row>
@@ -2644,8 +2711,8 @@
       <c r="F24" t="str">
         <v>IDFB0081813</v>
       </c>
-      <c r="G24" t="str">
-        <v>09/05/2026</v>
+      <c r="G24" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H24" t="str">
         <v>N</v>
@@ -2717,6 +2784,9 @@
         <v/>
       </c>
       <c r="AE24" t="str">
+        <v/>
+      </c>
+      <c r="AF24" t="str">
         <v/>
       </c>
     </row>
@@ -2739,8 +2809,8 @@
       <c r="F25" t="str">
         <v>IDFB0081813</v>
       </c>
-      <c r="G25" t="str">
-        <v>09/05/2026</v>
+      <c r="G25" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H25" t="str">
         <v>N</v>
@@ -2812,6 +2882,9 @@
         <v/>
       </c>
       <c r="AE25" t="str">
+        <v/>
+      </c>
+      <c r="AF25" t="str">
         <v/>
       </c>
     </row>
@@ -2834,8 +2907,8 @@
       <c r="F26" t="str">
         <v>IDFB0081813</v>
       </c>
-      <c r="G26" t="str">
-        <v>09/05/2026</v>
+      <c r="G26" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H26" t="str">
         <v>N</v>
@@ -2907,6 +2980,9 @@
         <v/>
       </c>
       <c r="AE26" t="str">
+        <v/>
+      </c>
+      <c r="AF26" t="str">
         <v/>
       </c>
     </row>
@@ -2929,8 +3005,8 @@
       <c r="F27" t="str">
         <v>ICIC0006310</v>
       </c>
-      <c r="G27" t="str">
-        <v>09/05/2026</v>
+      <c r="G27" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H27" t="str">
         <v>N</v>
@@ -3002,6 +3078,9 @@
         <v/>
       </c>
       <c r="AE27" t="str">
+        <v/>
+      </c>
+      <c r="AF27" t="str">
         <v/>
       </c>
     </row>
@@ -3024,8 +3103,8 @@
       <c r="F28" t="str">
         <v>ICIC0006310</v>
       </c>
-      <c r="G28" t="str">
-        <v>09/05/2026</v>
+      <c r="G28" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H28" t="str">
         <v>N</v>
@@ -3097,6 +3176,9 @@
         <v/>
       </c>
       <c r="AE28" t="str">
+        <v/>
+      </c>
+      <c r="AF28" t="str">
         <v/>
       </c>
     </row>
@@ -3119,8 +3201,8 @@
       <c r="F29" t="str">
         <v>ICIC0006310</v>
       </c>
-      <c r="G29" t="str">
-        <v>09/05/2026</v>
+      <c r="G29" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H29" t="str">
         <v>N</v>
@@ -3192,6 +3274,9 @@
         <v/>
       </c>
       <c r="AE29" t="str">
+        <v/>
+      </c>
+      <c r="AF29" t="str">
         <v/>
       </c>
     </row>
@@ -3214,8 +3299,8 @@
       <c r="F30" t="str">
         <v>UTIB0002070</v>
       </c>
-      <c r="G30" t="str">
-        <v>09/05/2026</v>
+      <c r="G30" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H30" t="str">
         <v>I</v>
@@ -3287,6 +3372,9 @@
         <v/>
       </c>
       <c r="AE30" t="str">
+        <v/>
+      </c>
+      <c r="AF30" t="str">
         <v/>
       </c>
     </row>
@@ -3309,8 +3397,8 @@
       <c r="F31" t="str">
         <v>SBIN0000055</v>
       </c>
-      <c r="G31" t="str">
-        <v>09/05/2026</v>
+      <c r="G31" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H31" t="str">
         <v>N</v>
@@ -3382,6 +3470,9 @@
         <v/>
       </c>
       <c r="AE31" t="str">
+        <v/>
+      </c>
+      <c r="AF31" t="str">
         <v/>
       </c>
     </row>
@@ -3404,8 +3495,8 @@
       <c r="F32" t="str">
         <v>UTIB0000029</v>
       </c>
-      <c r="G32" t="str">
-        <v>09/05/2026</v>
+      <c r="G32" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H32" t="str">
         <v>I</v>
@@ -3477,6 +3568,9 @@
         <v/>
       </c>
       <c r="AE32" t="str">
+        <v/>
+      </c>
+      <c r="AF32" t="str">
         <v/>
       </c>
     </row>
@@ -3499,8 +3593,8 @@
       <c r="F33" t="str">
         <v>UTIB0000029</v>
       </c>
-      <c r="G33" t="str">
-        <v>09/05/2026</v>
+      <c r="G33" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H33" t="str">
         <v>I</v>
@@ -3572,6 +3666,9 @@
         <v/>
       </c>
       <c r="AE33" t="str">
+        <v/>
+      </c>
+      <c r="AF33" t="str">
         <v/>
       </c>
     </row>
@@ -3594,8 +3691,8 @@
       <c r="F34" t="str">
         <v>ICIC0000169</v>
       </c>
-      <c r="G34" t="str">
-        <v>09/05/2026</v>
+      <c r="G34" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H34" t="str">
         <v>N</v>
@@ -3667,6 +3764,9 @@
         <v/>
       </c>
       <c r="AE34" t="str">
+        <v/>
+      </c>
+      <c r="AF34" t="str">
         <v/>
       </c>
     </row>
@@ -3689,8 +3789,8 @@
       <c r="F35" t="str">
         <v>UTIB0000029</v>
       </c>
-      <c r="G35" t="str">
-        <v>09/05/2026</v>
+      <c r="G35" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H35" t="str">
         <v>I</v>
@@ -3762,6 +3862,9 @@
         <v/>
       </c>
       <c r="AE35" t="str">
+        <v/>
+      </c>
+      <c r="AF35" t="str">
         <v/>
       </c>
     </row>
@@ -3784,8 +3887,8 @@
       <c r="F36" t="str">
         <v>UTIB0000029</v>
       </c>
-      <c r="G36" t="str">
-        <v>09/05/2026</v>
+      <c r="G36" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H36" t="str">
         <v>I</v>
@@ -3857,6 +3960,9 @@
         <v/>
       </c>
       <c r="AE36" t="str">
+        <v/>
+      </c>
+      <c r="AF36" t="str">
         <v/>
       </c>
     </row>
@@ -3879,8 +3985,8 @@
       <c r="F37" t="str">
         <v>UTIB0000029</v>
       </c>
-      <c r="G37" t="str">
-        <v>09/05/2026</v>
+      <c r="G37" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H37" t="str">
         <v>I</v>
@@ -3952,6 +4058,9 @@
         <v/>
       </c>
       <c r="AE37" t="str">
+        <v/>
+      </c>
+      <c r="AF37" t="str">
         <v/>
       </c>
     </row>
@@ -3974,8 +4083,8 @@
       <c r="F38" t="str">
         <v>UTIB0000029</v>
       </c>
-      <c r="G38" t="str">
-        <v>09/05/2026</v>
+      <c r="G38" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H38" t="str">
         <v>I</v>
@@ -4047,6 +4156,9 @@
         <v/>
       </c>
       <c r="AE38" t="str">
+        <v/>
+      </c>
+      <c r="AF38" t="str">
         <v/>
       </c>
     </row>
@@ -4069,8 +4181,8 @@
       <c r="F39" t="str">
         <v>UTIB0000029</v>
       </c>
-      <c r="G39" t="str">
-        <v>09/05/2026</v>
+      <c r="G39" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H39" t="str">
         <v>I</v>
@@ -4142,6 +4254,9 @@
         <v/>
       </c>
       <c r="AE39" t="str">
+        <v/>
+      </c>
+      <c r="AF39" t="str">
         <v/>
       </c>
     </row>
@@ -4164,8 +4279,8 @@
       <c r="F40" t="str">
         <v>UTIB0000029</v>
       </c>
-      <c r="G40" t="str">
-        <v>09/05/2026</v>
+      <c r="G40" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H40" t="str">
         <v>I</v>
@@ -4237,6 +4352,9 @@
         <v/>
       </c>
       <c r="AE40" t="str">
+        <v/>
+      </c>
+      <c r="AF40" t="str">
         <v/>
       </c>
     </row>
@@ -4259,8 +4377,8 @@
       <c r="F41" t="str">
         <v>HDFC0002870</v>
       </c>
-      <c r="G41" t="str">
-        <v>09/05/2026</v>
+      <c r="G41" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H41" t="str">
         <v>N</v>
@@ -4332,6 +4450,9 @@
         <v/>
       </c>
       <c r="AE41" t="str">
+        <v/>
+      </c>
+      <c r="AF41" t="str">
         <v/>
       </c>
     </row>
@@ -4354,8 +4475,8 @@
       <c r="F42" t="str">
         <v>CNRB0005566</v>
       </c>
-      <c r="G42" t="str">
-        <v>09/05/2026</v>
+      <c r="G42" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H42" t="str">
         <v>N</v>
@@ -4427,6 +4548,9 @@
         <v/>
       </c>
       <c r="AE42" t="str">
+        <v/>
+      </c>
+      <c r="AF42" t="str">
         <v/>
       </c>
     </row>
@@ -4449,8 +4573,8 @@
       <c r="F43" t="str">
         <v>CNRB0005566</v>
       </c>
-      <c r="G43" t="str">
-        <v>09/05/2026</v>
+      <c r="G43" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H43" t="str">
         <v>N</v>
@@ -4522,6 +4646,9 @@
         <v/>
       </c>
       <c r="AE43" t="str">
+        <v/>
+      </c>
+      <c r="AF43" t="str">
         <v/>
       </c>
     </row>
@@ -4544,8 +4671,8 @@
       <c r="F44" t="str">
         <v>CNRB0005566</v>
       </c>
-      <c r="G44" t="str">
-        <v>09/05/2026</v>
+      <c r="G44" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H44" t="str">
         <v>N</v>
@@ -4617,6 +4744,9 @@
         <v/>
       </c>
       <c r="AE44" t="str">
+        <v/>
+      </c>
+      <c r="AF44" t="str">
         <v/>
       </c>
     </row>
@@ -4639,8 +4769,8 @@
       <c r="F45" t="str">
         <v>CNRB0005566</v>
       </c>
-      <c r="G45" t="str">
-        <v>09/05/2026</v>
+      <c r="G45" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H45" t="str">
         <v>N</v>
@@ -4712,6 +4842,9 @@
         <v/>
       </c>
       <c r="AE45" t="str">
+        <v/>
+      </c>
+      <c r="AF45" t="str">
         <v/>
       </c>
     </row>
@@ -4734,8 +4867,8 @@
       <c r="F46" t="str">
         <v>CNRB0005566</v>
       </c>
-      <c r="G46" t="str">
-        <v>09/05/2026</v>
+      <c r="G46" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H46" t="str">
         <v>N</v>
@@ -4807,6 +4940,9 @@
         <v/>
       </c>
       <c r="AE46" t="str">
+        <v/>
+      </c>
+      <c r="AF46" t="str">
         <v/>
       </c>
     </row>
@@ -4829,8 +4965,8 @@
       <c r="F47" t="str">
         <v>ICIC0000169</v>
       </c>
-      <c r="G47" t="str">
-        <v>09/05/2026</v>
+      <c r="G47" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H47" t="str">
         <v>N</v>
@@ -4902,6 +5038,9 @@
         <v/>
       </c>
       <c r="AE47" t="str">
+        <v/>
+      </c>
+      <c r="AF47" t="str">
         <v/>
       </c>
     </row>
@@ -4924,8 +5063,8 @@
       <c r="F48" t="str">
         <v>SBIN0000572</v>
       </c>
-      <c r="G48" t="str">
-        <v>09/05/2026</v>
+      <c r="G48" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H48" t="str">
         <v>N</v>
@@ -4997,6 +5136,9 @@
         <v/>
       </c>
       <c r="AE48" t="str">
+        <v/>
+      </c>
+      <c r="AF48" t="str">
         <v/>
       </c>
     </row>
@@ -5019,8 +5161,8 @@
       <c r="F49" t="str">
         <v>CNRB0013128</v>
       </c>
-      <c r="G49" t="str">
-        <v>09/05/2026</v>
+      <c r="G49" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H49" t="str">
         <v>N</v>
@@ -5092,6 +5234,9 @@
         <v/>
       </c>
       <c r="AE49" t="str">
+        <v/>
+      </c>
+      <c r="AF49" t="str">
         <v/>
       </c>
     </row>
@@ -5114,8 +5259,8 @@
       <c r="F50" t="str">
         <v>HDFC0000592</v>
       </c>
-      <c r="G50" t="str">
-        <v>09/05/2026</v>
+      <c r="G50" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H50" t="str">
         <v>N</v>
@@ -5187,6 +5332,9 @@
         <v/>
       </c>
       <c r="AE50" t="str">
+        <v/>
+      </c>
+      <c r="AF50" t="str">
         <v/>
       </c>
     </row>
@@ -5209,8 +5357,8 @@
       <c r="F51" t="str">
         <v>HDFC0000592</v>
       </c>
-      <c r="G51" t="str">
-        <v>09/05/2026</v>
+      <c r="G51" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H51" t="str">
         <v>N</v>
@@ -5282,6 +5430,9 @@
         <v/>
       </c>
       <c r="AE51" t="str">
+        <v/>
+      </c>
+      <c r="AF51" t="str">
         <v/>
       </c>
     </row>
@@ -5304,8 +5455,8 @@
       <c r="F52" t="str">
         <v>HDFC0000592</v>
       </c>
-      <c r="G52" t="str">
-        <v>09/05/2026</v>
+      <c r="G52" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H52" t="str">
         <v>N</v>
@@ -5377,6 +5528,9 @@
         <v/>
       </c>
       <c r="AE52" t="str">
+        <v/>
+      </c>
+      <c r="AF52" t="str">
         <v/>
       </c>
     </row>
@@ -5399,8 +5553,8 @@
       <c r="F53" t="str">
         <v>HDFC0000212</v>
       </c>
-      <c r="G53" t="str">
-        <v>09/05/2026</v>
+      <c r="G53" s="2" t="str">
+        <v>05/09/2026</v>
       </c>
       <c r="H53" t="str">
         <v>N</v>
@@ -5472,13 +5626,16 @@
         <v/>
       </c>
       <c r="AE53" t="str">
+        <v/>
+      </c>
+      <c r="AF53" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AE53"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AF53"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Payment Mode to IMPS
</commit_message>
<xml_diff>
--- a/public/AxisBank_Payout_Verification.xlsx
+++ b/public/AxisBank_Payout_Verification.xlsx
@@ -559,7 +559,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H2" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I2" t="str">
         <v>PAY20260831658011</v>
@@ -657,7 +657,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H3" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I3" t="str">
         <v>PAY20260808003115</v>
@@ -755,7 +755,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H4" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I4" t="str">
         <v>PAY20260805061816</v>
@@ -853,7 +853,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H5" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I5" t="str">
         <v>PAY20260805059908</v>
@@ -951,7 +951,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H6" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I6" t="str">
         <v>PAY20260804613052</v>
@@ -1049,7 +1049,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H7" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I7" t="str">
         <v>PAY20260804046652</v>
@@ -1245,7 +1245,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H9" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I9" t="str">
         <v>PAY20260804375695</v>
@@ -1343,7 +1343,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H10" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I10" t="str">
         <v>PAY20260804451179</v>
@@ -1441,7 +1441,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H11" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I11" t="str">
         <v>PAY20260804546420</v>
@@ -1539,7 +1539,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H12" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I12" t="str">
         <v>PAY20260804405930</v>
@@ -1637,7 +1637,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H13" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I13" t="str">
         <v>PAY20260802315857</v>
@@ -1735,7 +1735,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H14" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I14" t="str">
         <v>PAY20260801933762</v>
@@ -1833,7 +1833,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H15" t="str">
-        <v>R</v>
+        <v>I</v>
       </c>
       <c r="I15" t="str">
         <v>PAY20260801762336</v>
@@ -1931,7 +1931,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H16" t="str">
-        <v>R</v>
+        <v>I</v>
       </c>
       <c r="I16" t="str">
         <v>PAY20260731875317</v>
@@ -2029,7 +2029,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H17" t="str">
-        <v>R</v>
+        <v>I</v>
       </c>
       <c r="I17" t="str">
         <v>PAY20260731912652</v>
@@ -2127,7 +2127,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H18" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I18" t="str">
         <v>PAY20260731523707</v>
@@ -2225,7 +2225,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H19" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I19" t="str">
         <v>PAY20260731578132</v>
@@ -2323,7 +2323,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H20" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I20" t="str">
         <v>PAY20260730226073</v>
@@ -2421,7 +2421,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H21" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I21" t="str">
         <v>PAY20260730913804</v>
@@ -2519,7 +2519,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H22" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I22" t="str">
         <v>PAY20260730456908</v>
@@ -2617,7 +2617,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H23" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I23" t="str">
         <v>PAY20260730386586</v>
@@ -2715,7 +2715,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H24" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I24" t="str">
         <v>PAY20260729419157</v>
@@ -2813,7 +2813,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H25" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I25" t="str">
         <v>PAY20260729438891</v>
@@ -2911,7 +2911,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H26" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I26" t="str">
         <v>PAY20260729580331</v>
@@ -3009,7 +3009,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H27" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I27" t="str">
         <v>PAY20260729383214</v>
@@ -3107,7 +3107,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H28" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I28" t="str">
         <v>PAY20260729258687</v>
@@ -3205,7 +3205,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H29" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I29" t="str">
         <v>PAY20260729476921</v>
@@ -3401,7 +3401,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H31" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I31" t="str">
         <v>PAY20260729529558</v>
@@ -3695,7 +3695,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H34" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I34" t="str">
         <v>PAY20260721460795</v>
@@ -4381,7 +4381,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H41" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I41" t="str">
         <v>PAY20260711958193</v>
@@ -4479,7 +4479,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H42" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I42" t="str">
         <v>PAY20260708826638</v>
@@ -4577,7 +4577,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H43" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I43" t="str">
         <v>PAY20260708863377</v>
@@ -4675,7 +4675,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H44" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I44" t="str">
         <v>PAY20260708320378</v>
@@ -4773,7 +4773,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H45" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I45" t="str">
         <v>PAY20260708088577</v>
@@ -4871,7 +4871,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H46" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I46" t="str">
         <v>PAY20260708050762</v>
@@ -4969,7 +4969,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H47" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I47" t="str">
         <v>PAY20260707269449</v>
@@ -5067,7 +5067,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H48" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I48" t="str">
         <v>PAY20260701805832</v>
@@ -5165,7 +5165,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H49" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I49" t="str">
         <v>PAY20260701319443</v>
@@ -5263,7 +5263,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H50" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I50" t="str">
         <v>PAY20260616951859</v>
@@ -5361,7 +5361,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H51" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I51" t="str">
         <v>PAY20260616469779</v>
@@ -5459,7 +5459,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H52" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I52" t="str">
         <v>PAY20260616172942</v>
@@ -5557,7 +5557,7 @@
         <v>05/09/2026</v>
       </c>
       <c r="H53" t="str">
-        <v>N</v>
+        <v>I</v>
       </c>
       <c r="I53" t="str">
         <v>PAY20260616639105</v>

</xml_diff>